<commit_message>
docs: ajustes de documentacao
</commit_message>
<xml_diff>
--- a/templates/pnl-forecast.xlsx
+++ b/templates/pnl-forecast.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="R9b28d9611b4743fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rddc2aee0d4454b1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" r:id="Rdbc56b09d95148bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="4" r:id="R3130045ca85544a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance" sheetId="5" r:id="Ref2b61aa2f7e4c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R5cc9ba4ccc8745ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R9a2db54396d141e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" r:id="Re6f7858b99874009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Ra1b02e2091b54f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" r:id="R4d7736de5dd24bba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="4" r:id="Rbc12b44bd9454985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variance" sheetId="5" r:id="R81ff9cb7c5f64c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="6" r:id="R8a6ea03c8bba4bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R3e6b0d0079554f97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -205,6 +205,21 @@
     <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -216,7 +231,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -227,7 +242,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -238,7 +253,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -448,126 +463,126 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>P&amp;L e Rolling Forecast — Operação Brasil</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="5" t="str">
-        <x:v>Purpose</x:v>
+        <x:v>Resultado e previsão contínua — Operação Brasil</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="39" t="str">
+        <x:v>Objetivo</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>Modelar base/upside/downside e variações mensais para decisão executiva.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="5" t="str">
-        <x:v>Version</x:v>
+        <x:v>Modelar cenários base, favorável e adverso e variações mensais para decidir.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="39" t="str">
+        <x:v>Versão</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
         <x:v>1.0</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="5" t="str">
-        <x:v>As of</x:v>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="39" t="str">
+        <x:v>Data de referência</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="5" t="str">
-        <x:v>Currency / scale</x:v>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="39" t="str">
+        <x:v>Moeda / escala</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>BRL thousands</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="5" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>R$ mil</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="39" t="str">
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>Jan-2026 to Dec-2027, monthly</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="5" t="str">
-        <x:v>Scenario</x:v>
+        <x:v>Jan/2026 a dez/2027, mensal</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="39" t="str">
+        <x:v>Cenário</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>Selector on Assumptions sheet</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="5" t="str">
-        <x:v>Color convention</x:v>
+        <x:v>Seletor na aba Assumptions (premissas)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="39" t="str">
+        <x:v>Convenção de cores</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>Blue font = input; black = formula; green = cross-sheet link.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="5" t="str">
-        <x:v>Model status</x:v>
+        <x:v>Azul: entrada; preto: fórmula; verde: vínculo entre abas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="39" t="str">
+        <x:v>Situação do modelo</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>See Checks sheet.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="5" t="str">
-        <x:v>Use</x:v>
+        <x:v>Ver aba Checks (verificações).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="39" t="str">
+        <x:v>Uso</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Synthetic teaching case; not target-company economics.</x:v>
+        <x:v>Caso didático sintético; não representa a economia da empresa estudada.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -590,77 +605,77 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Assumptions</x:v>
+        <x:v>Premissas</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Assumptions</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Driver</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Value</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="str">
-        <x:v>Unit</x:v>
-      </x:c>
-      <x:c r="D4" s="14" t="str">
-        <x:v>Note</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Scenario selector</x:v>
+        <x:v>Premissas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Premissa</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Unidade</x:v>
+      </x:c>
+      <x:c r="D4" s="42" t="str">
+        <x:v>Nota</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>Seletor de cenário</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
         <x:v>Base</x:v>
       </x:c>
-      <x:c r="C5" t="str">
-        <x:v>Base/Upside/Downside</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
-        <x:v>Editable</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>Initial self-serve revenue</x:v>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Base / Upside (favorável) / Downside (adverso)</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Editável</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Receita inicial por autosserviço</x:v>
       </x:c>
       <x:c r="B6" s="16" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="C6" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Monthly self-serve growth</x:v>
+      <x:c r="C6" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>Crescimento mensal por autosserviço</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:v>0.08</x:v>
@@ -668,27 +683,27 @@
       <x:c r="C7" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D7" t="str">
-        <x:v>before churn</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Initial enterprise revenue</x:v>
+      <x:c r="D7" s="6" t="str">
+        <x:v>antes das perdas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Receita empresarial inicial</x:v>
       </x:c>
       <x:c r="B8" s="16" t="n">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="C8" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>Monthly enterprise growth</x:v>
+      <x:c r="C8" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>Crescimento empresarial mensal</x:v>
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:v>0.1</x:v>
@@ -696,13 +711,13 @@
       <x:c r="C9" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D9" t="str">
-        <x:v>before churn</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Monthly revenue churn</x:v>
+      <x:c r="D9" s="6" t="str">
+        <x:v>antes das perdas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>Perda mensal de receita</x:v>
       </x:c>
       <x:c r="B10" s="17" t="n">
         <x:v>0.02</x:v>
@@ -710,13 +725,13 @@
       <x:c r="C10" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D10" t="str">
-        <x:v>applied to prior revenue</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>COGS % revenue</x:v>
+      <x:c r="D10" s="6" t="str">
+        <x:v>aplicado à receita anterior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>Custo dos serviços / receita</x:v>
       </x:c>
       <x:c r="B11" s="17" t="n">
         <x:v>0.28</x:v>
@@ -724,27 +739,27 @@
       <x:c r="C11" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D11" t="str">
-        <x:v>includes workload/support in teaching model</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Initial payroll</x:v>
+      <x:c r="D11" s="6" t="str">
+        <x:v>inclui carga de trabalho e suporte no modelo didático</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>Folha salarial inicial</x:v>
       </x:c>
       <x:c r="B12" s="16" t="n">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="C12" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>Monthly payroll growth</x:v>
+      <x:c r="C12" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>Crescimento mensal da folha</x:v>
       </x:c>
       <x:c r="B13" s="17" t="n">
         <x:v>0.03</x:v>
@@ -752,27 +767,27 @@
       <x:c r="C13" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D13" t="str">
-        <x:v>hiring/ramp proxy</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Initial non-payroll opex</x:v>
+      <x:c r="D13" s="6" t="str">
+        <x:v>aproximação de contratação/adaptação</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>Despesas operacionais iniciais sem folha</x:v>
       </x:c>
       <x:c r="B14" s="16" t="n">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="C14" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>Monthly non-payroll growth</x:v>
+      <x:c r="C14" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>Crescimento mensal de despesas sem folha</x:v>
       </x:c>
       <x:c r="B15" s="17" t="n">
         <x:v>0.01</x:v>
@@ -780,50 +795,50 @@
       <x:c r="C15" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="D15" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>Initial cash</x:v>
+      <x:c r="D15" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>Caixa inicial</x:v>
       </x:c>
       <x:c r="B16" s="16" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="C16" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>HQ funding month</x:v>
+      <x:c r="C16" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>Mês do aporte da matriz</x:v>
       </x:c>
       <x:c r="B17" s="16" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C17" t="str">
-        <x:v>month index</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>Synthetic</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>HQ funding amount</x:v>
+      <x:c r="C17" s="6" t="str">
+        <x:v>índice do mês</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Sintético</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>Valor do aporte da matriz</x:v>
       </x:c>
       <x:c r="B18" s="16" t="n">
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="C18" t="str">
-        <x:v>BRL k</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>Synthetic</x:v>
+      <x:c r="C18" s="6" t="str">
+        <x:v>R$ mil</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>Sintético</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -853,65 +868,65 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
+        <x:v>Multiplicadores por cenário</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>Scenario Multipliers</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Scenario</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Revenue growth</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="str">
-        <x:v>Churn</x:v>
-      </x:c>
-      <x:c r="D4" s="13" t="str">
-        <x:v>COGS</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="str">
-        <x:v>Payroll</x:v>
-      </x:c>
-      <x:c r="F4" s="14" t="str">
-        <x:v>Non-payroll</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>Multiplicadores por cenário</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Cenário</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Crescimento da receita</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Perda de receita</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>Custo dos serviços</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>Folha salarial</x:v>
+      </x:c>
+      <x:c r="F4" s="42" t="str">
+        <x:v>Demais despesas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" t="str">
         <x:v>Base</x:v>
       </x:c>
@@ -931,7 +946,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" t="str">
         <x:v>Upside</x:v>
       </x:c>
@@ -951,7 +966,7 @@
         <x:v>1.05</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" t="str">
         <x:v>Downside</x:v>
       </x:c>
@@ -1012,161 +1027,161 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="N1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="U1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="V1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="W1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="X1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="Y1" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="M2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="N2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="O2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="R2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="S2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="U2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="V2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="W2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="X2" s="3" t="str">
-        <x:v>Forecast</x:v>
+        <x:v>Previsão</x:v>
       </x:c>
       <x:c r="Y2" s="3" t="str">
-        <x:v>Forecast</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Line item</x:v>
+        <x:v>Previsão</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Linha</x:v>
       </x:c>
       <x:c r="B4" s="25" t="n">
         <x:v>46023</x:v>
@@ -1241,9 +1256,10 @@
         <x:v>46722</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>Self-serve revenue before churn</x:v>
+    <x:row r="5"/>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Receita por autosserviço antes das perdas</x:v>
       </x:c>
       <x:c r="B6" s="28" t="n">
         <x:f>'Assumptions'!$B$6</x:f>
@@ -1342,9 +1358,9 @@
         <x:v>1174.2927291185401</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Enterprise revenue before churn</x:v>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>Receita empresarial antes das perdas</x:v>
       </x:c>
       <x:c r="B7" s="28" t="n">
         <x:f>'Assumptions'!$B$8</x:f>
@@ -1443,9 +1459,9 @@
         <x:v>3581.720973020956</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Revenue churn</x:v>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Perda de receita</x:v>
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:f>-('Assumptions'!$B$6+'Assumptions'!$B$8)*'Assumptions'!$B$10*IF('Assumptions'!$B$5="Upside",'Scenarios'!$C$6,IF('Assumptions'!$B$5="Downside",'Scenarios'!$C$7,'Scenarios'!$C$5))</x:f>
@@ -1544,9 +1560,9 @@
         <x:v>-85.31007998272428</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="32" t="str">
-        <x:v>Total revenue</x:v>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="43" t="str">
+        <x:v>Receita total</x:v>
       </x:c>
       <x:c r="B9" s="33" t="n">
         <x:f>SUM(B6:B8)</x:f>
@@ -1645,9 +1661,9 @@
         <x:v>4670.703622156772</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>COGS</x:v>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>Custo dos serviços</x:v>
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>-B9*'Assumptions'!$B$11*IF('Assumptions'!$B$5="Upside",'Scenarios'!$D$6,IF('Assumptions'!$B$5="Downside",'Scenarios'!$D$7,'Scenarios'!$D$5))</x:f>
@@ -1746,9 +1762,9 @@
         <x:v>-1307.7970142038964</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="32" t="str">
-        <x:v>Gross profit</x:v>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="43" t="str">
+        <x:v>Lucro bruto</x:v>
       </x:c>
       <x:c r="B11" s="33" t="n">
         <x:f>SUM(B9:B10)</x:f>
@@ -1847,9 +1863,9 @@
         <x:v>3362.9066079528757</x:v>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>Gross margin</x:v>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>Margem bruta</x:v>
       </x:c>
       <x:c r="B12" s="29" t="n">
         <x:f>IF(B9=0,0,B11/B9)</x:f>
@@ -1948,9 +1964,9 @@
         <x:v>0.7199999999999999</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>Payroll</x:v>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>Folha salarial</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
         <x:f>-'Assumptions'!$B$12*IF('Assumptions'!$B$5="Upside",'Scenarios'!$E$6,IF('Assumptions'!$B$5="Downside",'Scenarios'!$E$7,'Scenarios'!$E$5))</x:f>
@@ -2049,9 +2065,9 @@
         <x:v>-769.6987393393761</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Non-payroll opex</x:v>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>Despesas operacionais sem folha</x:v>
       </x:c>
       <x:c r="B14" s="28" t="n">
         <x:f>-'Assumptions'!$B$14*IF('Assumptions'!$B$5="Upside",'Scenarios'!$F$6,IF('Assumptions'!$B$5="Downside",'Scenarios'!$F$7,'Scenarios'!$F$5))</x:f>
@@ -2150,9 +2166,9 @@
         <x:v>-326.862384770592</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="32" t="str">
-        <x:v>Total opex</x:v>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="43" t="str">
+        <x:v>Despesas operacionais totais</x:v>
       </x:c>
       <x:c r="B15" s="33" t="n">
         <x:f>SUM(B13:B14)</x:f>
@@ -2251,9 +2267,9 @@
         <x:v>-1096.561124109968</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="32" t="str">
-        <x:v>Operating income</x:v>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="43" t="str">
+        <x:v>Resultado operacional</x:v>
       </x:c>
       <x:c r="B16" s="33" t="n">
         <x:f>SUM(B11,B15)</x:f>
@@ -2352,9 +2368,9 @@
         <x:v>2266.345483842908</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>Operating margin</x:v>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>Margem operacional</x:v>
       </x:c>
       <x:c r="B17" s="29" t="n">
         <x:f>IF(B9=0,0,B16/B9)</x:f>
@@ -2453,9 +2469,9 @@
         <x:v>0.4852257105528752</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>HQ funding</x:v>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>Financiamento da matriz</x:v>
       </x:c>
       <x:c r="B18" s="28" t="n">
         <x:f>IF(COLUMN()-1='Assumptions'!$B$17,'Assumptions'!$B$18,0)</x:f>
@@ -2554,9 +2570,9 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>Net cash flow</x:v>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>Fluxo líquido de caixa</x:v>
       </x:c>
       <x:c r="B19" s="28" t="n">
         <x:f>SUM(B16,B18)</x:f>
@@ -2655,9 +2671,9 @@
         <x:v>2266.345483842908</x:v>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>Beginning cash</x:v>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>Caixa inicial</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
         <x:f>'Assumptions'!$B$16</x:f>
@@ -2756,9 +2772,9 @@
         <x:v>21764.7925894766</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="32" t="str">
-        <x:v>Ending cash</x:v>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="43" t="str">
+        <x:v>Caixa final</x:v>
       </x:c>
       <x:c r="B21" s="33" t="n">
         <x:f>SUM(B19:B20)</x:f>
@@ -2886,128 +2902,128 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
+        <x:v>Análise de desvios — realizado e previsão</x:v>
       </x:c>
       <x:c r="M2" s="3" t="str">
-        <x:v>Variance Analysis — Actual vs Forecast</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Month</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Actual revenue</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="str">
-        <x:v>Forecast revenue</x:v>
-      </x:c>
-      <x:c r="D4" s="13" t="str">
-        <x:v>Var BRL k</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="str">
-        <x:v>Var %</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="str">
-        <x:v>Actual COGS</x:v>
-      </x:c>
-      <x:c r="G4" s="13" t="str">
-        <x:v>Forecast COGS</x:v>
-      </x:c>
-      <x:c r="H4" s="13" t="str">
-        <x:v>Var COGS</x:v>
-      </x:c>
-      <x:c r="I4" s="13" t="str">
-        <x:v>Actual opex</x:v>
-      </x:c>
-      <x:c r="J4" s="13" t="str">
-        <x:v>Forecast opex</x:v>
-      </x:c>
-      <x:c r="K4" s="13" t="str">
-        <x:v>Var opex</x:v>
-      </x:c>
-      <x:c r="L4" s="13" t="str">
-        <x:v>Comment / driver</x:v>
-      </x:c>
-      <x:c r="M4" s="14" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>Análise de desvios — realizado e previsão</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Mês</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Receita realizada</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Receita prevista</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>Desvio em R$ mil</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>Desvio %</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="str">
+        <x:v>Custo realizado dos serviços</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="str">
+        <x:v>Custo previsto dos serviços</x:v>
+      </x:c>
+      <x:c r="H4" s="41" t="str">
+        <x:v>Desvio no custo dos serviços</x:v>
+      </x:c>
+      <x:c r="I4" s="41" t="str">
+        <x:v>Despesa operacional realizada</x:v>
+      </x:c>
+      <x:c r="J4" s="41" t="str">
+        <x:v>Despesa operacional prevista</x:v>
+      </x:c>
+      <x:c r="K4" s="41" t="str">
+        <x:v>Desvio em despesas operacionais</x:v>
+      </x:c>
+      <x:c r="L4" s="41" t="str">
+        <x:v>Comentário / causa</x:v>
+      </x:c>
+      <x:c r="M4" s="42" t="str">
+        <x:v>Responsável</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="19" t="n">
         <x:v>46023</x:v>
       </x:c>
@@ -3049,11 +3065,11 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L5" s="38" t="str"/>
-      <x:c r="M5" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="M5" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="19" t="n">
         <x:v>46054</x:v>
       </x:c>
@@ -3095,11 +3111,11 @@
         <x:v>5.7000000000000455</x:v>
       </x:c>
       <x:c r="L6" s="38" t="str"/>
-      <x:c r="M6" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+      <x:c r="M6" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="19" t="n">
         <x:v>46082</x:v>
       </x:c>
@@ -3141,11 +3157,11 @@
         <x:v>11.023000000000025</x:v>
       </x:c>
       <x:c r="L7" s="38" t="str"/>
-      <x:c r="M7" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+      <x:c r="M7" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="19" t="n">
         <x:v>46113</x:v>
       </x:c>
@@ -3187,11 +3203,11 @@
         <x:v>15.958210000000008</x:v>
       </x:c>
       <x:c r="L8" s="38" t="str"/>
-      <x:c r="M8" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+      <x:c r="M8" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="19" t="n">
         <x:v>46143</x:v>
       </x:c>
@@ -3233,11 +3249,11 @@
         <x:v>20.49452150000002</x:v>
       </x:c>
       <x:c r="L9" s="38" t="str"/>
-      <x:c r="M9" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+      <x:c r="M9" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="19" t="n">
         <x:v>46174</x:v>
       </x:c>
@@ -3279,11 +3295,11 @@
         <x:v>24.62049799700003</x:v>
       </x:c>
       <x:c r="L10" s="38" t="str"/>
-      <x:c r="M10" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
+      <x:c r="M10" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="19" t="n">
         <x:v>46204</x:v>
       </x:c>
@@ -3325,11 +3341,11 @@
         <x:v>38.32436519742987</x:v>
       </x:c>
       <x:c r="L11" s="38" t="str"/>
-      <x:c r="M11" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="M11" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="19" t="n">
         <x:v>46235</x:v>
       </x:c>
@@ -3371,11 +3387,11 @@
         <x:v>51.594000936478096</x:v>
       </x:c>
       <x:c r="L12" s="38" t="str"/>
-      <x:c r="M12" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
+      <x:c r="M12" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="19" t="n">
         <x:v>46266</x:v>
       </x:c>
@@ -3417,11 +3433,11 @@
         <x:v>64.41692479552876</x:v>
       </x:c>
       <x:c r="L13" s="38" t="str"/>
-      <x:c r="M13" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
+      <x:c r="M13" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="19" t="n">
         <x:v>46296</x:v>
       </x:c>
@@ -3463,11 +3479,11 @@
         <x:v>76.78028740866068</x:v>
       </x:c>
       <x:c r="L14" s="38" t="str"/>
-      <x:c r="M14" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
+      <x:c r="M14" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="19" t="n">
         <x:v>46327</x:v>
       </x:c>
@@ -3509,11 +3525,11 @@
         <x:v>88.67085944887913</x:v>
       </x:c>
       <x:c r="L15" s="38" t="str"/>
-      <x:c r="M15" s="16" t="str">
-        <x:v>Learner</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
+      <x:c r="M15" s="38" t="str">
+        <x:v>Participante</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="19" t="n">
         <x:v>46357</x:v>
       </x:c>
@@ -3555,8 +3571,8 @@
         <x:v>100.0750202844838</x:v>
       </x:c>
       <x:c r="L16" s="38" t="str"/>
-      <x:c r="M16" s="16" t="str">
-        <x:v>Learner</x:v>
+      <x:c r="M16" s="38" t="str">
+        <x:v>Participante</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3582,76 +3598,76 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>Checks</x:v>
+        <x:v>Verificações</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Checks</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>Check</x:v>
-      </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Actual</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="str">
-        <x:v>Expected</x:v>
-      </x:c>
-      <x:c r="D4" s="13" t="str">
-        <x:v>Difference</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="str">
-        <x:v>Tolerance</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="G4" s="14" t="str">
-        <x:v>Where to fix</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Scenario selector valid</x:v>
+        <x:v>Verificações</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Verificação</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Realizado</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Esperado</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>Diferença</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>Tolerância</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="str">
+        <x:v>Situação</x:v>
+      </x:c>
+      <x:c r="G4" s="42" t="str">
+        <x:v>Onde corrigir</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>Seletor de cenário válido</x:v>
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF('Scenarios'!A5:A7,'Assumptions'!B5)</x:f>
@@ -3675,9 +3691,9 @@
         <x:v>Assumptions B5</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>Revenue components tie final month</x:v>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Componentes da receita reconciliados no mês final</x:v>
       </x:c>
       <x:c r="B6" t="n">
         <x:f>'Forecast'!Y9</x:f>
@@ -3702,9 +3718,9 @@
         <x:v>Forecast rows 6:9</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Gross profit ties final month</x:v>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>Lucro bruto reconciliado no mês final</x:v>
       </x:c>
       <x:c r="B7" t="n">
         <x:f>'Forecast'!Y11</x:f>
@@ -3729,9 +3745,9 @@
         <x:v>Forecast rows 9:11</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Ending cash roll-forward ties</x:v>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Movimentação do caixa final reconciliada</x:v>
       </x:c>
       <x:c r="B8" t="n">
         <x:f>'Forecast'!Y21</x:f>
@@ -3756,16 +3772,16 @@
         <x:v>Forecast rows 19:21</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>MODEL STATUS</x:v>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>SITUAÇÃO DO MODELO</x:v>
       </x:c>
       <x:c r="F9" t="str">
         <x:f>IF(COUNTIF(F5:F8,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="G9" t="str">
-        <x:v>All checks</x:v>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Todas as verificações</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3799,133 +3815,133 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
+        <x:v>Fontes / auditoria</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Sources / Audit</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>Fontes / auditoria</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
         <x:v>Item</x:v>
       </x:c>
-      <x:c r="B4" s="13" t="str">
-        <x:v>Value</x:v>
-      </x:c>
-      <x:c r="C4" s="13" t="str">
-        <x:v>Units</x:v>
-      </x:c>
-      <x:c r="D4" s="13" t="str">
-        <x:v>Period / as-of</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="str">
-        <x:v>Source type</x:v>
-      </x:c>
-      <x:c r="F4" s="13" t="str">
-        <x:v>Source name</x:v>
+      <x:c r="B4" s="41" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C4" s="41" t="str">
+        <x:v>Unidades</x:v>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:v>Período / data de referência</x:v>
+      </x:c>
+      <x:c r="E4" s="41" t="str">
+        <x:v>Tipo da fonte</x:v>
+      </x:c>
+      <x:c r="F4" s="41" t="str">
+        <x:v>Nome da fonte</x:v>
       </x:c>
       <x:c r="G4" s="13" t="str">
         <x:v>URL</x:v>
       </x:c>
-      <x:c r="H4" s="13" t="str">
-        <x:v>Owner</x:v>
-      </x:c>
-      <x:c r="I4" s="13" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="J4" s="14" t="str">
-        <x:v>Accessed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="H4" s="41" t="str">
+        <x:v>Responsável</x:v>
+      </x:c>
+      <x:c r="I4" s="41" t="str">
+        <x:v>Notas</x:v>
+      </x:c>
+      <x:c r="J4" s="42" t="str">
+        <x:v>Consulta declarada</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>Scenario</x:v>
+        <x:v>Cenário</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>All financial inputs</x:v>
+        <x:v>Todos os dados financeiros</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
-        <x:v>BRL k</x:v>
+        <x:v>R$ mil</x:v>
       </x:c>
       <x:c r="D5" s="6" t="str">
         <x:v>2026-2027</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
-        <x:v>Synthetic</x:v>
+        <x:v>Sintético</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>M1 teaching case</x:v>
+        <x:v>Caso didático M1</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str"/>
       <x:c r="H5" s="6" t="str">
-        <x:v>Learner</x:v>
+        <x:v>Participante</x:v>
       </x:c>
       <x:c r="I5" s="6" t="str">
-        <x:v>Not target-company economics</x:v>
+        <x:v>Não representa a economia da empresa estudada</x:v>
       </x:c>
       <x:c r="J5" s="6" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="6" t="str">
-        <x:v>Consumption model comparison</x:v>
+        <x:v>Comparação de modelo por consumo</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
         <x:v>Snowflake FY2026 10-K</x:v>
@@ -3946,27 +3962,27 @@
         <x:v>https://www.sec.gov/Archives/edgar/data/1640147/000164014726000008/snow-20260131.htm</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str">
-        <x:v>Program</x:v>
+        <x:v>Programa</x:v>
       </x:c>
       <x:c r="I6" s="6" t="str">
-        <x:v>Conceptual comparison only</x:v>
+        <x:v>Comparação somente conceitual</x:v>
       </x:c>
       <x:c r="J6" s="6" t="str">
         <x:v>2026-07-23</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="6" t="str">
-        <x:v>FX reference</x:v>
+        <x:v>Referência cambial</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>Official exchange-rate resources</x:v>
+        <x:v>Fontes oficiais de câmbio</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>various</x:v>
+        <x:v>diversos</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>current</x:v>
+        <x:v>atual</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
         <x:v>T0</x:v>
@@ -3978,10 +3994,10 @@
         <x:v>https://www.bcb.gov.br/estabilidadefinanceira/cambioecapitais</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>Learner</x:v>
+        <x:v>Participante</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
-        <x:v>Use actual deal rate for real model</x:v>
+        <x:v>Usar câmbio contratado no modelo real</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
         <x:v>2026-07-23</x:v>

</xml_diff>